<commit_message>
Improve GCard report WOE rendering
</commit_message>
<xml_diff>
--- a/projects/2026-05-fujie-gcard-v1/versions/fujie_gcard_v7_20260630/reports_tuned_main_lgbm_tuned_balanced/model_report.xlsx
+++ b/projects/2026-05-fujie-gcard-v1/versions/fujie_gcard_v7_20260630/reports_tuned_main_lgbm_tuned_balanced/model_report.xlsx
@@ -35607,7 +35607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35622,1222 +35622,1189 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>3、意愿交叉风险（DEV-OOS）</t>
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>以下矩阵均限定 DEV-OOS；意愿评级按对应客群、对应分数版本等频三等分，资产评级为 zc_level 1-7，并保留行列合计。</t>
         </is>
       </c>
       <c r="B1" s="5" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>序号</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>结论</t>
-        </is>
-      </c>
-    </row>
+      <c r="C1" s="5" t="n"/>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="5" t="n"/>
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="5" t="n"/>
+      <c r="H1" s="5" t="n"/>
+    </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="7" t="n">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>老户 DEV-OOS 意愿 x 资产评级</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>老户 - 占比 - G卡V7</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>意愿</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>低意愿</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>0.0112092862092862</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>0.0551282051282051</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>0.0894317394317394</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>0.101039501039501</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>0.0136001386001386</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>0.0522695772695772</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.0106548856548856</v>
+      </c>
+      <c r="I7" s="15" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>中意愿</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>0.0141198891198891</v>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>0.0514553014553014</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>0.0638600138600138</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>0.0867983367983368</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>0.0154712404712404</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>0.0758316008316008</v>
+      </c>
+      <c r="H8" s="15" t="n">
+        <v>0.0257969507969507</v>
+      </c>
+      <c r="I8" s="15" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>高意愿</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>0.0126645876645876</v>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>0.0452356202356202</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>0.0629244629244629</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>0.08880803880803879</v>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>0.0149688149688149</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>0.0788981288981289</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>0.0298336798336798</v>
+      </c>
+      <c r="I9" s="15" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>0.0379937629937629</v>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>0.1518191268191268</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>0.2162162162162162</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>0.2766458766458766</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>0.044040194040194</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>0.206999306999307</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <v>0.0662855162855162</v>
+      </c>
+      <c r="I10" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>（1）高、中、低意愿评级为对应模型分数在各客群内三等频分箱得到。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>以下矩阵均限定 DEV-OOS；意愿评级按对应客群、对应分数版本等频三等分，资产评级为 zc_level 1-7，并保留行列合计。</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-    </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>老户 DEV-OOS 意愿 x 资产评级</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>老户 - 占比 - G卡V7</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>老户 - 30天发起率 - G卡V7</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>意愿</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>低意愿</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="n">
-        <v>0.0112092862092862</v>
-      </c>
-      <c r="C12" s="15" t="n">
-        <v>0.0551282051282051</v>
-      </c>
-      <c r="D12" s="15" t="n">
-        <v>0.0894317394317394</v>
-      </c>
-      <c r="E12" s="15" t="n">
-        <v>0.101039501039501</v>
-      </c>
-      <c r="F12" s="15" t="n">
-        <v>0.0136001386001386</v>
-      </c>
-      <c r="G12" s="15" t="n">
-        <v>0.0522695772695772</v>
-      </c>
-      <c r="H12" s="15" t="n">
-        <v>0.0106548856548856</v>
-      </c>
-      <c r="I12" s="15" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>中意愿</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="n">
-        <v>0.0141198891198891</v>
-      </c>
-      <c r="C13" s="15" t="n">
-        <v>0.0514553014553014</v>
-      </c>
-      <c r="D13" s="15" t="n">
-        <v>0.0638600138600138</v>
-      </c>
-      <c r="E13" s="15" t="n">
-        <v>0.0867983367983368</v>
-      </c>
-      <c r="F13" s="15" t="n">
-        <v>0.0154712404712404</v>
-      </c>
-      <c r="G13" s="15" t="n">
-        <v>0.0758316008316008</v>
-      </c>
-      <c r="H13" s="15" t="n">
-        <v>0.0257969507969507</v>
-      </c>
-      <c r="I13" s="15" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>高意愿</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="n">
-        <v>0.0126645876645876</v>
-      </c>
-      <c r="C14" s="15" t="n">
-        <v>0.0452356202356202</v>
-      </c>
-      <c r="D14" s="15" t="n">
-        <v>0.0629244629244629</v>
-      </c>
-      <c r="E14" s="15" t="n">
-        <v>0.08880803880803879</v>
-      </c>
-      <c r="F14" s="15" t="n">
-        <v>0.0149688149688149</v>
-      </c>
-      <c r="G14" s="15" t="n">
-        <v>0.0788981288981289</v>
-      </c>
-      <c r="H14" s="15" t="n">
-        <v>0.0298336798336798</v>
-      </c>
-      <c r="I14" s="15" t="n">
-        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
+          <t>低意愿</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>0.1576506955177743</v>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>0.1407919547454431</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>0.1418055017435102</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>0.150034293552812</v>
+      </c>
+      <c r="F15" s="15" t="n">
+        <v>0.1503184713375796</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>0.1581040768975803</v>
+      </c>
+      <c r="H15" s="15" t="n">
+        <v>0.1560975609756097</v>
+      </c>
+      <c r="I15" s="15" t="n">
+        <v>0.148024948024948</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>中意愿</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>0.4159509202453987</v>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>0.4144781144781145</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>0.4232230059685296</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>0.417564870259481</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>0.458006718924972</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>0.4537354352296093</v>
+      </c>
+      <c r="H16" s="15" t="n">
+        <v>0.4412357286769644</v>
+      </c>
+      <c r="I16" s="15" t="n">
+        <v>0.43004158004158</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>高意愿</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="n">
+        <v>0.7578659370725034</v>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>0.795863653772501</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>0.7926762114537445</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>0.8055013655872025</v>
+      </c>
+      <c r="F17" s="15" t="n">
+        <v>0.7824074074074074</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>0.7749231444883619</v>
+      </c>
+      <c r="H17" s="15" t="n">
+        <v>0.7799070847851336</v>
+      </c>
+      <c r="I17" s="15" t="n">
+        <v>0.7893970893970894</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B15" s="15" t="n">
-        <v>0.0379937629937629</v>
-      </c>
-      <c r="C15" s="15" t="n">
-        <v>0.1518191268191268</v>
-      </c>
-      <c r="D15" s="15" t="n">
-        <v>0.2162162162162162</v>
-      </c>
-      <c r="E15" s="15" t="n">
-        <v>0.2766458766458766</v>
-      </c>
-      <c r="F15" s="15" t="n">
-        <v>0.044040194040194</v>
-      </c>
-      <c r="G15" s="15" t="n">
-        <v>0.206999306999307</v>
-      </c>
-      <c r="H15" s="15" t="n">
-        <v>0.0662855162855162</v>
-      </c>
-      <c r="I15" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>老户 - 30天发起率 - G卡V7</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="B18" s="15" t="n">
+        <v>0.4537163702690378</v>
+      </c>
+      <c r="C18" s="15" t="n">
+        <v>0.4287344516718019</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>0.4143429487179487</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>0.4443887775551102</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>0.473249409913454</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>0.5015065282892535</v>
+      </c>
+      <c r="H18" s="15" t="n">
+        <v>0.5478306325143754</v>
+      </c>
+      <c r="I18" s="15" t="n">
+        <v>0.4558212058212058</v>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>老户 - 新增订单3期金额逾期率 - G卡V7</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
+      <c r="H21" s="5" t="n"/>
+      <c r="I21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>意愿</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>低意愿</t>
-        </is>
-      </c>
-      <c r="B20" s="15" t="n">
-        <v>0.1576506955177743</v>
-      </c>
-      <c r="C20" s="15" t="n">
-        <v>0.1407919547454431</v>
-      </c>
-      <c r="D20" s="15" t="n">
-        <v>0.1418055017435102</v>
-      </c>
-      <c r="E20" s="15" t="n">
-        <v>0.150034293552812</v>
-      </c>
-      <c r="F20" s="15" t="n">
-        <v>0.1503184713375796</v>
-      </c>
-      <c r="G20" s="15" t="n">
-        <v>0.1581040768975803</v>
-      </c>
-      <c r="H20" s="15" t="n">
-        <v>0.1560975609756097</v>
-      </c>
-      <c r="I20" s="15" t="n">
-        <v>0.148024948024948</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>中意愿</t>
-        </is>
-      </c>
-      <c r="B21" s="15" t="n">
-        <v>0.4159509202453987</v>
-      </c>
-      <c r="C21" s="15" t="n">
-        <v>0.4144781144781145</v>
-      </c>
-      <c r="D21" s="15" t="n">
-        <v>0.4232230059685296</v>
-      </c>
-      <c r="E21" s="15" t="n">
-        <v>0.417564870259481</v>
-      </c>
-      <c r="F21" s="15" t="n">
-        <v>0.458006718924972</v>
-      </c>
-      <c r="G21" s="15" t="n">
-        <v>0.4537354352296093</v>
-      </c>
-      <c r="H21" s="15" t="n">
-        <v>0.4412357286769644</v>
-      </c>
-      <c r="I21" s="15" t="n">
-        <v>0.43004158004158</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>高意愿</t>
-        </is>
-      </c>
-      <c r="B22" s="15" t="n">
-        <v>0.7578659370725034</v>
-      </c>
-      <c r="C22" s="15" t="n">
-        <v>0.795863653772501</v>
-      </c>
-      <c r="D22" s="15" t="n">
-        <v>0.7926762114537445</v>
-      </c>
-      <c r="E22" s="15" t="n">
-        <v>0.8055013655872025</v>
-      </c>
-      <c r="F22" s="15" t="n">
-        <v>0.7824074074074074</v>
-      </c>
-      <c r="G22" s="15" t="n">
-        <v>0.7749231444883619</v>
-      </c>
-      <c r="H22" s="15" t="n">
-        <v>0.7799070847851336</v>
-      </c>
-      <c r="I22" s="15" t="n">
-        <v>0.7893970893970894</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
+          <t>低意愿</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n">
+        <v>0.0323087574838298</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>0.008611639625493399</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>0.039544904931394</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>0.0361334137107048</v>
+      </c>
+      <c r="F23" s="15" t="n">
+        <v>0.0136527193541979</v>
+      </c>
+      <c r="G23" s="15" t="n">
+        <v>0.035696434223038</v>
+      </c>
+      <c r="H23" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="15" t="n">
+        <v>0.0266553219567532</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>中意愿</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>0.0213400160825072</v>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>0.0227639202671805</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>0.0414493680214617</v>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>0.0446821452990801</v>
+      </c>
+      <c r="F24" s="15" t="n">
+        <v>0.0252495877164835</v>
+      </c>
+      <c r="G24" s="15" t="n">
+        <v>0.0503424868185618</v>
+      </c>
+      <c r="H24" s="15" t="n">
+        <v>0.0873597620425407</v>
+      </c>
+      <c r="I24" s="15" t="n">
+        <v>0.033209708967333</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>高意愿</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>0.0319419912200306</v>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>0.0369991653035138</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>0.0513274944846388</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>0.0584439853141064</v>
+      </c>
+      <c r="F25" s="15" t="n">
+        <v>0.09829677262143779</v>
+      </c>
+      <c r="G25" s="15" t="n">
+        <v>0.09251907667709471</v>
+      </c>
+      <c r="H25" s="15" t="n">
+        <v>0.0409060914137395</v>
+      </c>
+      <c r="I25" s="15" t="n">
+        <v>0.0489142762289343</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B23" s="15" t="n">
-        <v>0.4537163702690378</v>
-      </c>
-      <c r="C23" s="15" t="n">
-        <v>0.4287344516718019</v>
-      </c>
-      <c r="D23" s="15" t="n">
-        <v>0.4143429487179487</v>
-      </c>
-      <c r="E23" s="15" t="n">
-        <v>0.4443887775551102</v>
-      </c>
-      <c r="F23" s="15" t="n">
-        <v>0.473249409913454</v>
-      </c>
-      <c r="G23" s="15" t="n">
-        <v>0.5015065282892535</v>
-      </c>
-      <c r="H23" s="15" t="n">
-        <v>0.5478306325143754</v>
-      </c>
-      <c r="I23" s="15" t="n">
-        <v>0.4558212058212058</v>
-      </c>
-    </row>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>老户 - 新增订单3期金额逾期率 - G卡V7</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n"/>
-      <c r="C26" s="5" t="n"/>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="5" t="n"/>
-      <c r="I26" s="5" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="B26" s="15" t="n">
+        <v>0.029100256362737</v>
+      </c>
+      <c r="C26" s="15" t="n">
+        <v>0.0306205592399156</v>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>0.0475325380445715</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>0.0530715870367645</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>0.066624285479436</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <v>0.0777624539436802</v>
+      </c>
+      <c r="H26" s="15" t="n">
+        <v>0.0519544430035813</v>
+      </c>
+      <c r="I26" s="15" t="n">
+        <v>0.0428829038916342</v>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>流失户 DEV-OOS 意愿 x 资产评级</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n"/>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="5" t="n"/>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>流失户 - 占比 - G卡V7</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>意愿</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
+      <c r="I32" s="6" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>低意愿</t>
         </is>
       </c>
-      <c r="B28" s="15" t="n">
-        <v>0.0323087574838298</v>
-      </c>
-      <c r="C28" s="15" t="n">
-        <v>0.008611639625493399</v>
-      </c>
-      <c r="D28" s="15" t="n">
-        <v>0.039544904931394</v>
-      </c>
-      <c r="E28" s="15" t="n">
-        <v>0.0361334137107048</v>
-      </c>
-      <c r="F28" s="15" t="n">
-        <v>0.0136527193541979</v>
-      </c>
-      <c r="G28" s="15" t="n">
-        <v>0.035696434223038</v>
-      </c>
-      <c r="H28" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" s="15" t="n">
-        <v>0.0266553219567532</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="B33" s="15" t="n">
+        <v>2.54679740226665e-05</v>
+      </c>
+      <c r="C33" s="15" t="n">
+        <v>0.0002631690649008</v>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>0.0019695233244195</v>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>0.0052124453499724</v>
+      </c>
+      <c r="F33" s="15" t="n">
+        <v>0.0124029033490385</v>
+      </c>
+      <c r="G33" s="15" t="n">
+        <v>0.1477312279808141</v>
+      </c>
+      <c r="H33" s="15" t="n">
+        <v>0.1657285962901651</v>
+      </c>
+      <c r="I33" s="15" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>中意愿</t>
         </is>
       </c>
-      <c r="B29" s="15" t="n">
-        <v>0.0213400160825072</v>
-      </c>
-      <c r="C29" s="15" t="n">
-        <v>0.0227639202671805</v>
-      </c>
-      <c r="D29" s="15" t="n">
-        <v>0.0414493680214617</v>
-      </c>
-      <c r="E29" s="15" t="n">
-        <v>0.0446821452990801</v>
-      </c>
-      <c r="F29" s="15" t="n">
-        <v>0.0252495877164835</v>
-      </c>
-      <c r="G29" s="15" t="n">
-        <v>0.0503424868185618</v>
-      </c>
-      <c r="H29" s="15" t="n">
-        <v>0.0873597620425407</v>
-      </c>
-      <c r="I29" s="15" t="n">
-        <v>0.033209708967333</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="B34" s="15" t="n">
+        <v>0.0009168470648159</v>
+      </c>
+      <c r="C34" s="15" t="n">
+        <v>0.0044908527526635</v>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>0.0148478288552145</v>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>0.0177002419457532</v>
+      </c>
+      <c r="F34" s="15" t="n">
+        <v>0.0548834840188463</v>
+      </c>
+      <c r="G34" s="15" t="n">
+        <v>0.1834458168852668</v>
+      </c>
+      <c r="H34" s="15" t="n">
+        <v>0.0570482618107729</v>
+      </c>
+      <c r="I34" s="15" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>高意愿</t>
         </is>
       </c>
-      <c r="B30" s="15" t="n">
-        <v>0.0319419912200306</v>
-      </c>
-      <c r="C30" s="15" t="n">
-        <v>0.0369991653035138</v>
-      </c>
-      <c r="D30" s="15" t="n">
-        <v>0.0513274944846388</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>0.0584439853141064</v>
-      </c>
-      <c r="F30" s="15" t="n">
-        <v>0.09829677262143779</v>
-      </c>
-      <c r="G30" s="15" t="n">
-        <v>0.09251907667709471</v>
-      </c>
-      <c r="H30" s="15" t="n">
-        <v>0.0409060914137395</v>
-      </c>
-      <c r="I30" s="15" t="n">
-        <v>0.0489142762289343</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="B35" s="15" t="n">
+        <v>0.015170423192835</v>
+      </c>
+      <c r="C35" s="15" t="n">
+        <v>0.0358673967485886</v>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>0.0534742561229254</v>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>0.0344072329046224</v>
+      </c>
+      <c r="F35" s="15" t="n">
+        <v>0.0754106710811155</v>
+      </c>
+      <c r="G35" s="15" t="n">
+        <v>0.1032641453372384</v>
+      </c>
+      <c r="H35" s="15" t="n">
+        <v>0.0157392079460078</v>
+      </c>
+      <c r="I35" s="15" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B31" s="15" t="n">
-        <v>0.029100256362737</v>
-      </c>
-      <c r="C31" s="15" t="n">
-        <v>0.0306205592399156</v>
-      </c>
-      <c r="D31" s="15" t="n">
-        <v>0.0475325380445715</v>
-      </c>
-      <c r="E31" s="15" t="n">
-        <v>0.0530715870367645</v>
-      </c>
-      <c r="F31" s="15" t="n">
-        <v>0.066624285479436</v>
-      </c>
-      <c r="G31" s="15" t="n">
-        <v>0.0777624539436802</v>
-      </c>
-      <c r="H31" s="15" t="n">
-        <v>0.0519544430035813</v>
-      </c>
-      <c r="I31" s="15" t="n">
-        <v>0.0428829038916342</v>
-      </c>
-    </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34">
-      <c r="A34" s="13" t="inlineStr">
-        <is>
-          <t>流失户 DEV-OOS 意愿 x 资产评级</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="n"/>
-      <c r="C34" s="5" t="n"/>
-      <c r="D34" s="5" t="n"/>
-      <c r="E34" s="5" t="n"/>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="5" t="n"/>
-      <c r="H34" s="5" t="n"/>
-    </row>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>流失户 - 占比 - G卡V7</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="n"/>
-      <c r="C36" s="5" t="n"/>
-      <c r="D36" s="5" t="n"/>
-      <c r="E36" s="5" t="n"/>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="5" t="n"/>
-      <c r="I36" s="5" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+      <c r="B36" s="15" t="n">
+        <v>0.0161127382316736</v>
+      </c>
+      <c r="C36" s="15" t="n">
+        <v>0.040621418566153</v>
+      </c>
+      <c r="D36" s="15" t="n">
+        <v>0.0702916083025595</v>
+      </c>
+      <c r="E36" s="15" t="n">
+        <v>0.057319920200348</v>
+      </c>
+      <c r="F36" s="15" t="n">
+        <v>0.1426970584490003</v>
+      </c>
+      <c r="G36" s="15" t="n">
+        <v>0.4344411902033193</v>
+      </c>
+      <c r="H36" s="15" t="n">
+        <v>0.2385160660469459</v>
+      </c>
+      <c r="I36" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>流失户 - 30天发起率 - G卡V7</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n"/>
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="5" t="n"/>
+      <c r="I39" s="5" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>意愿</t>
         </is>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G40" s="6" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="H40" s="6" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I37" s="6" t="inlineStr">
+      <c r="I40" s="6" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>低意愿</t>
-        </is>
-      </c>
-      <c r="B38" s="15" t="n">
-        <v>2.54679740226665e-05</v>
-      </c>
-      <c r="C38" s="15" t="n">
-        <v>0.0002631690649008</v>
-      </c>
-      <c r="D38" s="15" t="n">
-        <v>0.0019695233244195</v>
-      </c>
-      <c r="E38" s="15" t="n">
-        <v>0.0052124453499724</v>
-      </c>
-      <c r="F38" s="15" t="n">
-        <v>0.0124029033490385</v>
-      </c>
-      <c r="G38" s="15" t="n">
-        <v>0.1477312279808141</v>
-      </c>
-      <c r="H38" s="15" t="n">
-        <v>0.1657285962901651</v>
-      </c>
-      <c r="I38" s="15" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>中意愿</t>
-        </is>
-      </c>
-      <c r="B39" s="15" t="n">
-        <v>0.0009168470648159</v>
-      </c>
-      <c r="C39" s="15" t="n">
-        <v>0.0044908527526635</v>
-      </c>
-      <c r="D39" s="15" t="n">
-        <v>0.0148478288552145</v>
-      </c>
-      <c r="E39" s="15" t="n">
-        <v>0.0177002419457532</v>
-      </c>
-      <c r="F39" s="15" t="n">
-        <v>0.0548834840188463</v>
-      </c>
-      <c r="G39" s="15" t="n">
-        <v>0.1834458168852668</v>
-      </c>
-      <c r="H39" s="15" t="n">
-        <v>0.0570482618107729</v>
-      </c>
-      <c r="I39" s="15" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>高意愿</t>
-        </is>
-      </c>
-      <c r="B40" s="15" t="n">
-        <v>0.015170423192835</v>
-      </c>
-      <c r="C40" s="15" t="n">
-        <v>0.0358673967485886</v>
-      </c>
-      <c r="D40" s="15" t="n">
-        <v>0.0534742561229254</v>
-      </c>
-      <c r="E40" s="15" t="n">
-        <v>0.0344072329046224</v>
-      </c>
-      <c r="F40" s="15" t="n">
-        <v>0.0754106710811155</v>
-      </c>
-      <c r="G40" s="15" t="n">
-        <v>0.1032641453372384</v>
-      </c>
-      <c r="H40" s="15" t="n">
-        <v>0.0157392079460078</v>
-      </c>
-      <c r="I40" s="15" t="n">
-        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
+          <t>低意愿</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="15" t="n">
+        <v>0.0043103448275862</v>
+      </c>
+      <c r="E41" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="15" t="n">
+        <v>0.0027378507871321</v>
+      </c>
+      <c r="G41" s="15" t="n">
+        <v>0.0021836570509136</v>
+      </c>
+      <c r="H41" s="15" t="n">
+        <v>0.0024075402110439</v>
+      </c>
+      <c r="I41" s="15" t="n">
+        <v>0.0022921176620399</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>中意愿</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="15" t="n">
+        <v>0.0075614366729678</v>
+      </c>
+      <c r="D42" s="15" t="n">
+        <v>0.006861063464837</v>
+      </c>
+      <c r="E42" s="15" t="n">
+        <v>0.0057553956834532</v>
+      </c>
+      <c r="F42" s="15" t="n">
+        <v>0.0061871616395978</v>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>0.0068952751168494</v>
+      </c>
+      <c r="H42" s="15" t="n">
+        <v>0.0083333333333333</v>
+      </c>
+      <c r="I42" s="15" t="n">
+        <v>0.0069527569081879</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>高意愿</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="n">
+        <v>0.0912143256855064</v>
+      </c>
+      <c r="C43" s="15" t="n">
+        <v>0.0752662721893491</v>
+      </c>
+      <c r="D43" s="15" t="n">
+        <v>0.0598507699634862</v>
+      </c>
+      <c r="E43" s="15" t="n">
+        <v>0.0523069331359486</v>
+      </c>
+      <c r="F43" s="15" t="n">
+        <v>0.0569627378138016</v>
+      </c>
+      <c r="G43" s="15" t="n">
+        <v>0.0752219664584018</v>
+      </c>
+      <c r="H43" s="15" t="n">
+        <v>0.1402373247033441</v>
+      </c>
+      <c r="I43" s="15" t="n">
+        <v>0.0700623965363555</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B41" s="15" t="n">
-        <v>0.0161127382316736</v>
-      </c>
-      <c r="C41" s="15" t="n">
-        <v>0.040621418566153</v>
-      </c>
-      <c r="D41" s="15" t="n">
-        <v>0.0702916083025595</v>
-      </c>
-      <c r="E41" s="15" t="n">
-        <v>0.057319920200348</v>
-      </c>
-      <c r="F41" s="15" t="n">
-        <v>0.1426970584490003</v>
-      </c>
-      <c r="G41" s="15" t="n">
-        <v>0.4344411902033193</v>
-      </c>
-      <c r="H41" s="15" t="n">
-        <v>0.2385160660469459</v>
-      </c>
-      <c r="I41" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>流失户 - 30天发起率 - G卡V7</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="n"/>
-      <c r="C44" s="5" t="n"/>
-      <c r="D44" s="5" t="n"/>
-      <c r="E44" s="5" t="n"/>
-      <c r="F44" s="5" t="n"/>
-      <c r="G44" s="5" t="n"/>
-      <c r="H44" s="5" t="n"/>
-      <c r="I44" s="5" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
+      <c r="B44" s="15" t="n">
+        <v>0.08587987355110641</v>
+      </c>
+      <c r="C44" s="15" t="n">
+        <v>0.06729362591431549</v>
+      </c>
+      <c r="D44" s="15" t="n">
+        <v>0.0471014492753623</v>
+      </c>
+      <c r="E44" s="15" t="n">
+        <v>0.0331753554502369</v>
+      </c>
+      <c r="F44" s="15" t="n">
+        <v>0.0327205663632577</v>
+      </c>
+      <c r="G44" s="15" t="n">
+        <v>0.021533952125061</v>
+      </c>
+      <c r="H44" s="15" t="n">
+        <v>0.0129199886104783</v>
+      </c>
+      <c r="I44" s="15" t="n">
+        <v>0.0264357570355278</v>
+      </c>
+    </row>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>流失户 - 新增订单3期金额逾期率 - G卡V7</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n"/>
+      <c r="C47" s="5" t="n"/>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="5" t="n"/>
+      <c r="F47" s="5" t="n"/>
+      <c r="G47" s="5" t="n"/>
+      <c r="H47" s="5" t="n"/>
+      <c r="I47" s="5" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>意愿</t>
         </is>
       </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F45" s="6" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="G45" s="6" t="inlineStr">
+      <c r="G48" s="6" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr">
+      <c r="H48" s="6" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I45" s="6" t="inlineStr">
+      <c r="I48" s="6" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>低意愿</t>
-        </is>
-      </c>
-      <c r="B46" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C46" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="15" t="n">
-        <v>0.0043103448275862</v>
-      </c>
-      <c r="E46" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="15" t="n">
-        <v>0.0027378507871321</v>
-      </c>
-      <c r="G46" s="15" t="n">
-        <v>0.0021836570509136</v>
-      </c>
-      <c r="H46" s="15" t="n">
-        <v>0.0024075402110439</v>
-      </c>
-      <c r="I46" s="15" t="n">
-        <v>0.0022921176620399</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>中意愿</t>
-        </is>
-      </c>
-      <c r="B47" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C47" s="15" t="n">
-        <v>0.0075614366729678</v>
-      </c>
-      <c r="D47" s="15" t="n">
-        <v>0.006861063464837</v>
-      </c>
-      <c r="E47" s="15" t="n">
-        <v>0.0057553956834532</v>
-      </c>
-      <c r="F47" s="15" t="n">
-        <v>0.0061871616395978</v>
-      </c>
-      <c r="G47" s="15" t="n">
-        <v>0.0068952751168494</v>
-      </c>
-      <c r="H47" s="15" t="n">
-        <v>0.0083333333333333</v>
-      </c>
-      <c r="I47" s="15" t="n">
-        <v>0.0069527569081879</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>高意愿</t>
-        </is>
-      </c>
-      <c r="B48" s="15" t="n">
-        <v>0.0912143256855064</v>
-      </c>
-      <c r="C48" s="15" t="n">
-        <v>0.0752662721893491</v>
-      </c>
-      <c r="D48" s="15" t="n">
-        <v>0.0598507699634862</v>
-      </c>
-      <c r="E48" s="15" t="n">
-        <v>0.0523069331359486</v>
-      </c>
-      <c r="F48" s="15" t="n">
-        <v>0.0569627378138016</v>
-      </c>
-      <c r="G48" s="15" t="n">
-        <v>0.0752219664584018</v>
-      </c>
-      <c r="H48" s="15" t="n">
-        <v>0.1402373247033441</v>
-      </c>
-      <c r="I48" s="15" t="n">
-        <v>0.0700623965363555</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
+          <t>低意愿</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>中意愿</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="15" t="n">
+        <v>0.0165774948875549</v>
+      </c>
+      <c r="E50" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="15" t="n">
+        <v>0.1714847347672421</v>
+      </c>
+      <c r="G50" s="15" t="n">
+        <v>0.1730771735522329</v>
+      </c>
+      <c r="H50" s="15" t="n">
+        <v>0.0286460007819287</v>
+      </c>
+      <c r="I50" s="15" t="n">
+        <v>0.1262030289119844</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>高意愿</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="n">
+        <v>0.0393828169465833</v>
+      </c>
+      <c r="C51" s="15" t="n">
+        <v>0.0512647772940201</v>
+      </c>
+      <c r="D51" s="15" t="n">
+        <v>0.0397594387590541</v>
+      </c>
+      <c r="E51" s="15" t="n">
+        <v>0.0184595915314542</v>
+      </c>
+      <c r="F51" s="15" t="n">
+        <v>0.0490848860098146</v>
+      </c>
+      <c r="G51" s="15" t="n">
+        <v>0.0490799977647711</v>
+      </c>
+      <c r="H51" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="15" t="n">
+        <v>0.0422069102478506</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B49" s="15" t="n">
-        <v>0.08587987355110641</v>
-      </c>
-      <c r="C49" s="15" t="n">
-        <v>0.06729362591431549</v>
-      </c>
-      <c r="D49" s="15" t="n">
-        <v>0.0471014492753623</v>
-      </c>
-      <c r="E49" s="15" t="n">
-        <v>0.0331753554502369</v>
-      </c>
-      <c r="F49" s="15" t="n">
-        <v>0.0327205663632577</v>
-      </c>
-      <c r="G49" s="15" t="n">
-        <v>0.021533952125061</v>
-      </c>
-      <c r="H49" s="15" t="n">
-        <v>0.0129199886104783</v>
-      </c>
-      <c r="I49" s="15" t="n">
-        <v>0.0264357570355278</v>
-      </c>
-    </row>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>流失户 - 新增订单3期金额逾期率 - G卡V7</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="n"/>
-      <c r="C52" s="5" t="n"/>
-      <c r="D52" s="5" t="n"/>
-      <c r="E52" s="5" t="n"/>
-      <c r="F52" s="5" t="n"/>
-      <c r="G52" s="5" t="n"/>
-      <c r="H52" s="5" t="n"/>
-      <c r="I52" s="5" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>意愿</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I53" s="6" t="inlineStr">
-        <is>
-          <t>合计</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>低意愿</t>
-        </is>
-      </c>
-      <c r="B54" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C54" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E54" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>中意愿</t>
-        </is>
-      </c>
-      <c r="B55" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C55" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="15" t="n">
-        <v>0.0165774948875549</v>
-      </c>
-      <c r="E55" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="15" t="n">
-        <v>0.1714847347672421</v>
-      </c>
-      <c r="G55" s="15" t="n">
-        <v>0.1730771735522329</v>
-      </c>
-      <c r="H55" s="15" t="n">
-        <v>0.0286460007819287</v>
-      </c>
-      <c r="I55" s="15" t="n">
-        <v>0.1262030289119844</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>高意愿</t>
-        </is>
-      </c>
-      <c r="B56" s="15" t="n">
+      <c r="B52" s="15" t="n">
         <v>0.0393828169465833</v>
       </c>
-      <c r="C56" s="15" t="n">
-        <v>0.0512647772940201</v>
-      </c>
-      <c r="D56" s="15" t="n">
-        <v>0.0397594387590541</v>
-      </c>
-      <c r="E56" s="15" t="n">
-        <v>0.0184595915314542</v>
-      </c>
-      <c r="F56" s="15" t="n">
-        <v>0.0490848860098146</v>
-      </c>
-      <c r="G56" s="15" t="n">
-        <v>0.0490799977647711</v>
-      </c>
-      <c r="H56" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I56" s="15" t="n">
-        <v>0.0422069102478506</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="7" t="inlineStr">
-        <is>
-          <t>合计</t>
-        </is>
-      </c>
-      <c r="B57" s="15" t="n">
-        <v>0.0393828169465833</v>
-      </c>
-      <c r="C57" s="15" t="n">
+      <c r="C52" s="15" t="n">
         <v>0.0511710568587837</v>
       </c>
-      <c r="D57" s="15" t="n">
+      <c r="D52" s="15" t="n">
         <v>0.0364962103504686</v>
       </c>
-      <c r="E57" s="15" t="n">
+      <c r="E52" s="15" t="n">
         <v>0.0179759421990095</v>
       </c>
-      <c r="F57" s="15" t="n">
+      <c r="F52" s="15" t="n">
         <v>0.0634558099772638</v>
       </c>
-      <c r="G57" s="15" t="n">
+      <c r="G52" s="15" t="n">
         <v>0.0763676785486706</v>
       </c>
-      <c r="H57" s="15" t="n">
+      <c r="H52" s="15" t="n">
         <v>0.0030933433616706</v>
       </c>
-      <c r="I57" s="15" t="n">
+      <c r="I52" s="15" t="n">
         <v>0.047161726640022</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A52:I52"/>
-    <mergeCell ref="A10:I10"/>
-    <mergeCell ref="A36:I36"/>
-    <mergeCell ref="A44:I44"/>
-    <mergeCell ref="A18:I18"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A34:H34"/>
+  <mergeCells count="9">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A39:I39"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A21:I21"/>
   </mergeCells>
-  <conditionalFormatting sqref="B12:I15">
+  <conditionalFormatting sqref="B7:I10">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -36849,7 +36816,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B20:I23">
+  <conditionalFormatting sqref="B15:I18">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -36861,7 +36828,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B28:I31">
+  <conditionalFormatting sqref="B23:I26">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -36873,7 +36840,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B38:I41">
+  <conditionalFormatting sqref="B33:I36">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -36885,7 +36852,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B46:I49">
+  <conditionalFormatting sqref="B41:I44">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -36897,7 +36864,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B54:I57">
+  <conditionalFormatting sqref="B49:I52">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>